<commit_message>
Switch published draft reports to the neutral public edition (no rating wording)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/reports/BAJFINANCE_NS_Financial_Model.xlsx
+++ b/public/reports/BAJFINANCE_NS_Financial_Model.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2321" uniqueCount="631">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2301" uniqueCount="623">
   <si>
     <t>Bajaj Finance Limited (BAJFINANCE.NS)</t>
   </si>
@@ -56,7 +56,7 @@
     <t>Fair value per share (INR)</t>
   </si>
   <si>
-    <t>Upside / (downside)</t>
+    <t>Model valuation spread vs price (an unaudited model output, not a rating; not independently audited)</t>
   </si>
   <si>
     <t>Primary method</t>
@@ -74,7 +74,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>Non-Banking Financial Company (NBFC) valued via RESIDUAL_INCOME_PB. 54/54 accounting invariants passed; reasonableness verdict ECONOMICALLY_SOUND.</t>
+    <t>Non-Banking Financial Company (NBFC) valued via RESIDUAL_INCOME_PB. 54/54 accounting invariants passed; reasonableness assessment ECONOMICALLY_SOUND.</t>
   </si>
   <si>
     <t>KEY FINANCIALS (₹ Crores)</t>
@@ -191,19 +191,19 @@
     <t>Snapshot ID</t>
   </si>
   <si>
-    <t>snap_BAJFINANCE_NS_84b3744f3a0e</t>
+    <t>snap_BAJFINANCE_NS_14a597949db9</t>
   </si>
   <si>
     <t>Snapshot SHA-256</t>
   </si>
   <si>
-    <t>84b3744f3a0e846d4706199ccdb856d784832a172b3e1ca66f301826a75875e3</t>
+    <t>14a597949db9912c1fbde077b91e080580c0a1d505ad2f73993429b3fce0ad91</t>
   </si>
   <si>
     <t>Built at</t>
   </si>
   <si>
-    <t>2026-11-01T14:58:21.687Z</t>
+    <t>2026-11-01T15:05:35.584Z</t>
   </si>
   <si>
     <t>Analysis status</t>
@@ -275,7 +275,7 @@
     <t>364.92</t>
   </si>
   <si>
-    <t>Upside / (downside) %</t>
+    <t>Model valuation spread vs price (an unaudited model output, not a rating; not independently audited) %</t>
   </si>
   <si>
     <t>-61.14</t>
@@ -761,7 +761,7 @@
     <t>DCF cross-check</t>
   </si>
   <si>
-    <t>Not eligible by methodology: valuation methodology routes this archetype (NBFC) to RESIDUAL_INCOME_PB and prohibits the consolidated FCFF DCF . It is not forced to populate a sheet, and no DCF stance is published.</t>
+    <t>Not eligible by methodology: valuation methodology routes this archetype (NBFC) to RESIDUAL_INCOME_PB and prohibits the consolidated FCFF DCF . It is not forced to populate a sheet, and no DCF reading is published.</t>
   </si>
   <si>
     <t>Segment analysis</t>
@@ -926,7 +926,7 @@
     <t>Withheld: Historical EPS (share basis) -- the statement share count (61.8 Cr) is 10.06x away from the valuation's 622 Cr, so FY24, FY25, FY26 EPS is withheld rather than shown on a basis the per-share fair value does not use. Confirm the dated split / bonus from the exchange record, then restate onto one basis.</t>
   </si>
   <si>
-    <t>Withheld: DCF cross-check -- Not eligible by methodology: valuation methodology routes this archetype (NBFC) to RESIDUAL_INCOME_PB and prohibits the consolidated FCFF DCF . It is not forced to populate a sheet, and no DCF stance is published.</t>
+    <t>Withheld: DCF cross-check -- Not eligible by methodology: valuation methodology routes this archetype (NBFC) to RESIDUAL_INCOME_PB and prohibits the consolidated FCFF DCF . It is not forced to populate a sheet, and no DCF reading is published.</t>
   </si>
   <si>
     <t>Withheld: Segment analysis -- no Ind AS 108 segment disclosure was read for this issuer and the provider published no split</t>
@@ -1124,7 +1124,7 @@
     <t>Forensic audit complete: Overall Health: UNAVAILABLE | Altman Z: N/A (N/A) | Piotroski F: N/A/9 | Beneish M: N/A (N/A).</t>
   </si>
   <si>
-    <t>ACCOUNTING QUALITY (verdict UNAVAILABLE)</t>
+    <t>ACCOUNTING QUALITY (assessment UNAVAILABLE)</t>
   </si>
   <si>
     <t>Check</t>
@@ -1598,40 +1598,16 @@
     <t>Assumptions hash (12)</t>
   </si>
   <si>
-    <t>snap_BAJFINANCE_NS_84b3744f3a0e  &lt;- THIS WORKBOOK</t>
+    <t>snap_BAJFINANCE_NS_14a597949db9  &lt;- THIS WORKBOOK</t>
   </si>
   <si>
     <t>74234e98afe7</t>
   </si>
   <si>
-    <t>snap_BAJFINANCE_NS_d356dbb4731b</t>
-  </si>
-  <si>
-    <t>2026-11-01T14:58:21.606Z</t>
-  </si>
-  <si>
-    <t>snap_BAJFINANCE_NS_79455fd41d7e</t>
-  </si>
-  <si>
-    <t>2026-11-01T14:56:25.526Z</t>
-  </si>
-  <si>
-    <t>snap_BAJFINANCE_NS_7fb5bf8ae42a</t>
-  </si>
-  <si>
-    <t>2026-11-01T14:56:25.431Z</t>
-  </si>
-  <si>
-    <t>snap_BAJFINANCE_NS_a2e6890202ad</t>
-  </si>
-  <si>
-    <t>2026-11-01T14:53:44.361Z</t>
-  </si>
-  <si>
-    <t>snap_BAJFINANCE_NS_18e0893cbcd1</t>
-  </si>
-  <si>
-    <t>2026-11-01T14:53:44.269Z</t>
+    <t>snap_BAJFINANCE_NS_9d96b80a9c43</t>
+  </si>
+  <si>
+    <t>2026-11-01T15:05:35.503Z</t>
   </si>
   <si>
     <t>OVERRIDES APPLIED TO THIS WORKBOOK</t>
@@ -1829,13 +1805,13 @@
     <t>a funding shortfall is withheld by the model, not published as negative borrowings or negative liquidity</t>
   </si>
   <si>
-    <t>No DCF stance without a DCF</t>
+    <t>No DCF reading without a DCF</t>
   </si>
   <si>
     <t>VALUATION</t>
   </si>
   <si>
-    <t>no DCF ran and no stance is published</t>
+    <t>no DCF ran and no reading is published</t>
   </si>
   <si>
     <t>No bonus / split is classified as economic dilution</t>
@@ -1916,7 +1892,7 @@
     <t>SAVED RECORD AND VERIFIER RECEIPTS</t>
   </si>
   <si>
-    <t>This snapshot's saved record (provenance, publication states, discrepancies, peer selection, limits and every verifier receipt) is kept by FMB beside the exported files: GET /api/export/snapshot/snap_BAJFINANCE_NS_84b3744f3a0e/record. Receipts are appended as verifiers run (workbook formula re-derivation, independent Monte Carlo), so they are read from the record, not stored in this file.</t>
+    <t>This snapshot's saved record (provenance, publication states, discrepancies, peer selection, limits and every verifier receipt) is kept by FMB beside the exported files: GET /api/export/snapshot/snap_BAJFINANCE_NS_14a597949db9/record. Receipts are appended as verifiers run (workbook formula re-derivation, independent Monte Carlo), so they are read from the record, not stored in this file.</t>
   </si>
   <si>
     <t>Chart data (editable)</t>
@@ -7853,7 +7829,7 @@
 
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I21"/>
+  <dimension ref="A1:I17"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="56" customWidth="1"/>
@@ -7974,208 +7950,84 @@
         <v>520</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
         <v>523</v>
       </c>
-      <c r="B8" t="s">
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
+      <c r="F9" s="4"/>
+      <c r="G9" s="4"/>
+      <c r="H9" s="4"/>
+      <c r="I9" s="4"/>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>524</v>
       </c>
-      <c r="C8" s="27">
-        <v>939.1</v>
-      </c>
-      <c r="D8" t="s">
-        <v>60</v>
-      </c>
-      <c r="E8" t="s">
-        <v>73</v>
-      </c>
-      <c r="F8" s="27">
-        <v>364.92</v>
-      </c>
-      <c r="G8" s="27">
-        <f>F8-364.92</f>
-        <v>0</v>
-      </c>
-      <c r="H8" s="33">
-        <f>G8/364.92</f>
-        <v>0</v>
-      </c>
-      <c r="I8" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" s="3" t="s">
         <v>525</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B12" s="4"/>
+      <c r="C12" s="4"/>
+      <c r="D12" s="4"/>
+      <c r="E12" s="4"/>
+      <c r="F12" s="4"/>
+      <c r="G12" s="4"/>
+      <c r="H12" s="4"/>
+      <c r="I12" s="4"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
         <v>526</v>
       </c>
-      <c r="C9" s="27">
-        <v>939.1</v>
-      </c>
-      <c r="D9" t="s">
-        <v>60</v>
-      </c>
-      <c r="E9" t="s">
-        <v>73</v>
-      </c>
-      <c r="F9" s="27">
-        <v>364.92</v>
-      </c>
-      <c r="G9" s="27">
-        <f>F9-364.92</f>
-        <v>0</v>
-      </c>
-      <c r="H9" s="33">
-        <f>G9/364.92</f>
-        <v>0</v>
-      </c>
-      <c r="I9" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="B13" t="s">
         <v>527</v>
       </c>
-      <c r="B10" t="s">
+      <c r="C13" t="s">
         <v>528</v>
       </c>
-      <c r="C10" s="27">
-        <v>939.1</v>
-      </c>
-      <c r="D10" t="s">
-        <v>60</v>
-      </c>
-      <c r="E10" t="s">
-        <v>73</v>
-      </c>
-      <c r="F10" s="27">
-        <v>364.92</v>
-      </c>
-      <c r="G10" s="27">
-        <f>F10-364.92</f>
-        <v>0</v>
-      </c>
-      <c r="H10" s="33">
-        <f>G10/364.92</f>
-        <v>0</v>
-      </c>
-      <c r="I10" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
         <v>529</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B14" t="s">
         <v>530</v>
       </c>
-      <c r="C11" s="27">
-        <v>939.1</v>
-      </c>
-      <c r="D11" t="s">
-        <v>60</v>
-      </c>
-      <c r="E11" t="s">
-        <v>73</v>
-      </c>
-      <c r="F11" s="27">
-        <v>364.92</v>
-      </c>
-      <c r="G11" s="27">
-        <f>F11-364.92</f>
-        <v>0</v>
-      </c>
-      <c r="H11" s="33">
-        <f>G11/364.92</f>
-        <v>0</v>
-      </c>
-      <c r="I11" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A13" s="3" t="s">
+      <c r="C14" t="s">
         <v>531</v>
       </c>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
-      <c r="I13" s="4"/>
-    </row>
-    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>526</v>
+      </c>
+      <c r="B15" t="s">
         <v>532</v>
       </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A16" s="3" t="s">
+      <c r="C15" t="s">
         <v>533</v>
       </c>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
-      <c r="I16" s="4"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>526</v>
+      </c>
+      <c r="B16" t="s">
         <v>534</v>
       </c>
-      <c r="B17" t="s">
+      <c r="C16" t="s">
         <v>535</v>
       </c>
-      <c r="C17" t="s">
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="2" t="s">
         <v>536</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>537</v>
-      </c>
-      <c r="B18" t="s">
-        <v>538</v>
-      </c>
-      <c r="C18" t="s">
-        <v>539</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>534</v>
-      </c>
-      <c r="B19" t="s">
-        <v>540</v>
-      </c>
-      <c r="C19" t="s">
-        <v>541</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>534</v>
-      </c>
-      <c r="B20" t="s">
-        <v>542</v>
-      </c>
-      <c r="C20" t="s">
-        <v>543</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.25">
-      <c r="A21" s="2" t="s">
-        <v>544</v>
       </c>
     </row>
   </sheetData>
@@ -8200,17 +8052,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>545</v>
+        <v>537</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>546</v>
+        <v>538</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>547</v>
+        <v>539</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -8222,7 +8074,7 @@
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="9" t="s">
-        <v>548</v>
+        <v>540</v>
       </c>
       <c r="B5" s="10" t="s">
         <v>451</v>
@@ -8234,27 +8086,27 @@
         <v>175</v>
       </c>
       <c r="E5" s="10" t="s">
-        <v>549</v>
+        <v>541</v>
       </c>
       <c r="F5" s="10" t="s">
         <v>8</v>
       </c>
       <c r="G5" s="10" t="s">
-        <v>550</v>
+        <v>542</v>
       </c>
       <c r="H5" s="10" t="s">
         <v>508</v>
       </c>
       <c r="I5" s="10" t="s">
-        <v>551</v>
+        <v>543</v>
       </c>
       <c r="J5" s="10" t="s">
-        <v>552</v>
+        <v>544</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>553</v>
+        <v>545</v>
       </c>
       <c r="B6" t="s">
         <v>459</v>
@@ -8263,19 +8115,19 @@
         <v>48319.6</v>
       </c>
       <c r="D6" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
       <c r="E6" t="s">
         <v>299</v>
       </c>
       <c r="F6" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="G6" t="s">
-        <v>556</v>
+        <v>548</v>
       </c>
       <c r="H6" t="s">
-        <v>557</v>
+        <v>549</v>
       </c>
       <c r="I6" t="s">
         <v>24</v>
@@ -8286,7 +8138,7 @@
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>558</v>
+        <v>550</v>
       </c>
       <c r="B7" t="s">
         <v>459</v>
@@ -8295,19 +8147,19 @@
         <v>14451.2</v>
       </c>
       <c r="D7" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
       <c r="E7" t="s">
         <v>299</v>
       </c>
       <c r="F7" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="G7" t="s">
-        <v>556</v>
+        <v>548</v>
       </c>
       <c r="H7" t="s">
-        <v>557</v>
+        <v>549</v>
       </c>
       <c r="I7" t="s">
         <v>24</v>
@@ -8318,7 +8170,7 @@
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>559</v>
+        <v>551</v>
       </c>
       <c r="B8" t="s">
         <v>486</v>
@@ -8327,19 +8179,19 @@
         <v>61204.9</v>
       </c>
       <c r="D8" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
       <c r="E8" t="s">
         <v>299</v>
       </c>
       <c r="F8" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="G8" t="s">
-        <v>560</v>
+        <v>552</v>
       </c>
       <c r="H8" t="s">
-        <v>561</v>
+        <v>553</v>
       </c>
       <c r="I8" t="s">
         <v>24</v>
@@ -8350,7 +8202,7 @@
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>562</v>
+        <v>554</v>
       </c>
       <c r="B9" t="s">
         <v>486</v>
@@ -8359,19 +8211,19 @@
         <v>16637.8</v>
       </c>
       <c r="D9" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
       <c r="E9" t="s">
         <v>299</v>
       </c>
       <c r="F9" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="G9" t="s">
-        <v>560</v>
+        <v>552</v>
       </c>
       <c r="H9" t="s">
-        <v>561</v>
+        <v>553</v>
       </c>
       <c r="I9" t="s">
         <v>24</v>
@@ -8382,7 +8234,7 @@
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>563</v>
+        <v>555</v>
       </c>
       <c r="B10" t="s">
         <v>494</v>
@@ -8391,19 +8243,19 @@
         <v>72783.1</v>
       </c>
       <c r="D10" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
       <c r="E10" t="s">
         <v>299</v>
       </c>
       <c r="F10" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="G10" t="s">
-        <v>564</v>
+        <v>556</v>
       </c>
       <c r="H10" t="s">
-        <v>565</v>
+        <v>557</v>
       </c>
       <c r="I10" t="s">
         <v>24</v>
@@ -8414,7 +8266,7 @@
     </row>
     <row r="11" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>566</v>
+        <v>558</v>
       </c>
       <c r="B11" t="s">
         <v>494</v>
@@ -8423,19 +8275,19 @@
         <v>19017.4</v>
       </c>
       <c r="D11" t="s">
-        <v>554</v>
+        <v>546</v>
       </c>
       <c r="E11" t="s">
         <v>299</v>
       </c>
       <c r="F11" t="s">
-        <v>555</v>
+        <v>547</v>
       </c>
       <c r="G11" t="s">
-        <v>564</v>
+        <v>556</v>
       </c>
       <c r="H11" t="s">
-        <v>565</v>
+        <v>557</v>
       </c>
       <c r="I11" t="s">
         <v>24</v>
@@ -8446,7 +8298,7 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>567</v>
+        <v>559</v>
       </c>
       <c r="B13" s="4"/>
       <c r="C13" s="4"/>
@@ -8461,19 +8313,19 @@
         <v>362</v>
       </c>
       <c r="B14" s="10" t="s">
-        <v>568</v>
+        <v>560</v>
       </c>
       <c r="C14" s="10" t="s">
         <v>10</v>
       </c>
       <c r="D14" s="10" t="s">
-        <v>569</v>
+        <v>561</v>
       </c>
       <c r="E14" s="10" t="s">
-        <v>570</v>
+        <v>562</v>
       </c>
       <c r="F14" s="10" t="s">
-        <v>571</v>
+        <v>563</v>
       </c>
       <c r="G14" s="10" t="s">
         <v>366</v>
@@ -8481,13 +8333,13 @@
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>572</v>
+        <v>564</v>
       </c>
       <c r="B15" t="s">
         <v>302</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>573</v>
+        <v>565</v>
       </c>
       <c r="D15" t="s">
         <v>24</v>
@@ -8499,18 +8351,18 @@
         <v>14.68</v>
       </c>
       <c r="G15" t="s">
-        <v>574</v>
+        <v>566</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>575</v>
+        <v>567</v>
       </c>
       <c r="B16" t="s">
         <v>302</v>
       </c>
       <c r="C16" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D16" t="s">
         <v>24</v>
@@ -8522,18 +8374,18 @@
         <v>0</v>
       </c>
       <c r="G16" t="s">
-        <v>577</v>
+        <v>569</v>
       </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>578</v>
+        <v>570</v>
       </c>
       <c r="B17" t="s">
         <v>302</v>
       </c>
       <c r="C17" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D17" t="s">
         <v>24</v>
@@ -8545,18 +8397,18 @@
         <v>0</v>
       </c>
       <c r="G17" t="s">
-        <v>579</v>
+        <v>571</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>580</v>
+        <v>572</v>
       </c>
       <c r="B18" t="s">
         <v>302</v>
       </c>
       <c r="C18" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D18" t="s">
         <v>24</v>
@@ -8568,18 +8420,18 @@
         <v>0</v>
       </c>
       <c r="G18" t="s">
-        <v>581</v>
+        <v>573</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>582</v>
+        <v>574</v>
       </c>
       <c r="B19" t="s">
         <v>302</v>
       </c>
       <c r="C19" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D19" t="s">
         <v>24</v>
@@ -8591,18 +8443,18 @@
         <v>0</v>
       </c>
       <c r="G19" t="s">
-        <v>583</v>
+        <v>575</v>
       </c>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>584</v>
+        <v>576</v>
       </c>
       <c r="B20" t="s">
         <v>302</v>
       </c>
       <c r="C20" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D20" t="s">
         <v>24</v>
@@ -8614,18 +8466,18 @@
         <v>0</v>
       </c>
       <c r="G20" t="s">
-        <v>585</v>
+        <v>577</v>
       </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>586</v>
+        <v>578</v>
       </c>
       <c r="B21" t="s">
         <v>302</v>
       </c>
       <c r="C21" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D21" t="s">
         <v>24</v>
@@ -8637,18 +8489,18 @@
         <v>0</v>
       </c>
       <c r="G21" t="s">
-        <v>587</v>
+        <v>579</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>588</v>
+        <v>580</v>
       </c>
       <c r="B22" t="s">
         <v>302</v>
       </c>
       <c r="C22" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D22" t="s">
         <v>24</v>
@@ -8660,18 +8512,18 @@
         <v>0</v>
       </c>
       <c r="G22" t="s">
-        <v>589</v>
+        <v>581</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>590</v>
+        <v>582</v>
       </c>
       <c r="B23" t="s">
         <v>302</v>
       </c>
       <c r="C23" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D23" t="s">
         <v>24</v>
@@ -8683,18 +8535,18 @@
         <v>0</v>
       </c>
       <c r="G23" t="s">
-        <v>591</v>
+        <v>583</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>592</v>
+        <v>584</v>
       </c>
       <c r="B24" t="s">
         <v>302</v>
       </c>
       <c r="C24" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D24" t="s">
         <v>24</v>
@@ -8706,18 +8558,18 @@
         <v>0</v>
       </c>
       <c r="G24" t="s">
-        <v>593</v>
+        <v>585</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>594</v>
+        <v>586</v>
       </c>
       <c r="B25" t="s">
         <v>302</v>
       </c>
       <c r="C25" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D25" t="s">
         <v>24</v>
@@ -8729,18 +8581,18 @@
         <v>0</v>
       </c>
       <c r="G25" t="s">
-        <v>595</v>
+        <v>587</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>596</v>
+        <v>588</v>
       </c>
       <c r="B26" t="s">
-        <v>597</v>
+        <v>589</v>
       </c>
       <c r="C26" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D26" t="s">
         <v>24</v>
@@ -8752,18 +8604,18 @@
         <v>24</v>
       </c>
       <c r="G26" t="s">
-        <v>598</v>
+        <v>590</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>599</v>
+        <v>591</v>
       </c>
       <c r="B27" t="s">
-        <v>600</v>
+        <v>592</v>
       </c>
       <c r="C27" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D27" t="s">
         <v>24</v>
@@ -8775,18 +8627,18 @@
         <v>24</v>
       </c>
       <c r="G27" t="s">
-        <v>601</v>
+        <v>593</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>602</v>
+        <v>594</v>
       </c>
       <c r="B28" t="s">
-        <v>603</v>
+        <v>595</v>
       </c>
       <c r="C28" t="s">
-        <v>576</v>
+        <v>568</v>
       </c>
       <c r="D28" t="s">
         <v>24</v>
@@ -8798,12 +8650,12 @@
         <v>24</v>
       </c>
       <c r="G28" t="s">
-        <v>604</v>
+        <v>596</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30" s="3" t="s">
-        <v>605</v>
+        <v>597</v>
       </c>
       <c r="B30" s="4"/>
       <c r="C30" s="4"/>
@@ -8815,41 +8667,41 @@
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="9" t="s">
-        <v>606</v>
+        <v>598</v>
       </c>
       <c r="B31" s="10" t="s">
-        <v>568</v>
+        <v>560</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>607</v>
+        <v>599</v>
       </c>
       <c r="D31" s="10" t="s">
-        <v>608</v>
+        <v>600</v>
       </c>
       <c r="E31" s="10" t="s">
-        <v>609</v>
+        <v>601</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>610</v>
+        <v>602</v>
       </c>
       <c r="B32" t="s">
-        <v>611</v>
+        <v>603</v>
       </c>
       <c r="C32" t="s">
-        <v>612</v>
+        <v>604</v>
       </c>
       <c r="D32" t="s">
         <v>248</v>
       </c>
       <c r="E32" t="s">
-        <v>613</v>
+        <v>605</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34" s="3" t="s">
-        <v>614</v>
+        <v>606</v>
       </c>
       <c r="B34" s="4"/>
       <c r="C34" s="4"/>
@@ -8861,10 +8713,10 @@
     </row>
     <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
-        <v>615</v>
+        <v>607</v>
       </c>
       <c r="B35" t="s">
-        <v>616</v>
+        <v>608</v>
       </c>
     </row>
     <row r="36" spans="1:2" x14ac:dyDescent="0.25">
@@ -8893,10 +8745,10 @@
     </row>
     <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
-        <v>617</v>
+        <v>609</v>
       </c>
       <c r="B39" t="s">
-        <v>618</v>
+        <v>610</v>
       </c>
     </row>
     <row r="40" spans="1:2" x14ac:dyDescent="0.25">
@@ -8904,12 +8756,12 @@
         <v>8</v>
       </c>
       <c r="B40" t="s">
-        <v>619</v>
+        <v>611</v>
       </c>
     </row>
     <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
-        <v>620</v>
+        <v>612</v>
       </c>
       <c r="B41" t="s">
         <v>229</v>
@@ -8917,7 +8769,7 @@
     </row>
     <row r="42" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
-        <v>621</v>
+        <v>613</v>
       </c>
       <c r="B42" t="s">
         <v>236</v>
@@ -8928,7 +8780,7 @@
     </row>
     <row r="43" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
-        <v>621</v>
+        <v>613</v>
       </c>
       <c r="B43" t="s">
         <v>239</v>
@@ -8939,7 +8791,7 @@
     </row>
     <row r="44" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
-        <v>621</v>
+        <v>613</v>
       </c>
       <c r="B44" t="s">
         <v>241</v>
@@ -8950,7 +8802,7 @@
     </row>
     <row r="45" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
-        <v>621</v>
+        <v>613</v>
       </c>
       <c r="B45" t="s">
         <v>243</v>
@@ -8961,15 +8813,15 @@
     </row>
     <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
-        <v>622</v>
+        <v>614</v>
       </c>
       <c r="B46" t="s">
-        <v>623</v>
+        <v>615</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48" s="3" t="s">
-        <v>624</v>
+        <v>616</v>
       </c>
       <c r="B48" s="4"/>
       <c r="C48" s="4"/>
@@ -8981,7 +8833,7 @@
     </row>
     <row r="49" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A49" s="2" t="s">
-        <v>625</v>
+        <v>617</v>
       </c>
     </row>
   </sheetData>
@@ -9001,17 +8853,17 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>626</v>
+        <v>618</v>
       </c>
     </row>
     <row r="2" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>627</v>
+        <v>619</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
-        <v>628</v>
+        <v>620</v>
       </c>
       <c r="B4" s="4"/>
       <c r="C4" s="4"/>
@@ -9021,12 +8873,12 @@
     </row>
     <row r="5" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>629</v>
+        <v>621</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" s="3" t="s">
-        <v>630</v>
+        <v>622</v>
       </c>
       <c r="B7" s="4"/>
       <c r="C7" s="4"/>

</xml_diff>